<commit_message>
feat: add dropdowns to excel input sheet template
- Scheme(s) column now uses Schemes lookup sheet as dropdown source
- Implementing Agency locked to BUIDCo via single-value dropdown
- CoS-EoT Log: Category column dropdown (Scope Addition, Scope Deletion, Design Change, Quantity Variation, Others)
- Management Actions Log: Status column dropdown (Open, Closed)
- Regenerated Template.xlsx with updated validations
- Updated package-lock.json files after npm install

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/src/assets/Template.xlsx
+++ b/frontend/src/assets/Template.xlsx
@@ -27,7 +27,7 @@
     <comment ref="H2" authorId="0">
       <text>
         <r>
-          <t>Comma-separated scheme names, e.g. "AMRUT 1.0, Namami Gange".</t>
+          <t>Pick from the Schemes sheet.</t>
         </r>
       </text>
     </comment>
@@ -145,7 +145,7 @@
     <t>CoS/EoT events, GeoTagging photos, and Management Action items each belong to a project but are entered from the Input Sheet directly after the project exists — the "…Log" sheets here are blank reference templates for jotting that data down by hand, not something this import reads.</t>
   </si>
   <si>
-    <t>Generated: 2026-09-02 11:46:57Z</t>
+    <t>Generated: 2026-10-03 10:09:27Z</t>
   </si>
   <si>
     <t>#</t>
@@ -1946,7 +1946,7 @@
         <v>98</v>
       </c>
       <c r="M3" s="16" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="N3" s="16" t="s">
         <v>103</v>
@@ -3128,7 +3128,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A2:BT2"/>
-  <dataValidations count="42">
+  <dataValidations count="44">
     <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a non-negative number (e.g. 12.5)." sqref="AA4:AA203">
       <formula1>0</formula1>
     </dataValidation>
@@ -3224,8 +3224,14 @@
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Pick a name from the Divisions sheet." sqref="E4:E203">
       <formula1>=Divisions!$A$2:$A$46</formula1>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Pick a name from the Schemes sheet." sqref="H4:H203">
+      <formula1>=Schemes!$A$2:$A$9</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Pick one of: Work Contract, Service Contract, O&amp;M Contract, Others" sqref="K4:K203">
       <formula1>"Work Contract,Service Contract,O&amp;M Contract,Others"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Pick one of: BUIDCo" sqref="M4:M203">
+      <formula1>"BUIDCo"</formula1>
     </dataValidation>
     <dataValidation type="date" operator="greaterThan" allowBlank="1" showErrorMessage="1" errorTitle="Invalid date" error="Enter a valid date (YYYY-MM-DD or use the Excel date picker)." sqref="N4:N203">
       <formula1>32874</formula1>
@@ -3315,6 +3321,11 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Pick one of: Scope Addition, Scope Deletion, Design Change, Quantity Variation, Others" sqref="D2:D201">
+      <formula1>"Scope Addition,Scope Deletion,Design Change,Quantity Variation,Others"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -3373,6 +3384,11 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Pick one of: Open, Closed" sqref="C2:C201">
+      <formula1>"Open,Closed"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>